<commit_message>
22 abril 2026 - estado actual app y fase6
</commit_message>
<xml_diff>
--- a/data/05_modelado/results/resultados_maestro.xlsx
+++ b/data/05_modelado/results/resultados_maestro.xlsx
@@ -527,43 +527,43 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.9318107808306586</v>
+        <v>0.9537035966611166</v>
       </c>
       <c r="E2" t="n">
-        <v>0.003240052843877967</v>
+        <v>0.001773359836655011</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7861853076417151</v>
+        <v>0.8317326001672022</v>
       </c>
       <c r="G2" t="n">
-        <v>0.004214369557038035</v>
+        <v>0.003983930847886074</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8485475672104397</v>
+        <v>0.874027598124419</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7326457993894749</v>
+        <v>0.7935408590485407</v>
       </c>
       <c r="J2" t="n">
-        <v>8.340999999999999</v>
+        <v>16.899</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9242</v>
+        <v>0.9573</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7645</v>
+        <v>0.8336</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8354</v>
+        <v>0.8692</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7046</v>
+        <v>0.8007</v>
       </c>
       <c r="O2" t="n">
-        <v>0.6784</v>
+        <v>0.7687</v>
       </c>
       <c r="P2" t="n">
-        <v>0.3026</v>
+        <v>0.2325</v>
       </c>
     </row>
     <row r="3">
@@ -574,52 +574,52 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.9314043328872905</v>
+        <v>0.9530835320729514</v>
       </c>
       <c r="E3" t="n">
-        <v>0.003268597955859321</v>
+        <v>0.002143235763700093</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7865254210379804</v>
+        <v>0.8259156953118418</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00404726089486917</v>
+        <v>0.00358620689183591</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8490216740390399</v>
+        <v>0.7935193910772284</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7329001713314985</v>
+        <v>0.8611740690867409</v>
       </c>
       <c r="J3" t="n">
-        <v>14.638</v>
+        <v>10.126</v>
       </c>
       <c r="K3" t="n">
-        <v>0.9263</v>
+        <v>0.9572000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7815</v>
+        <v>0.8298</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8456</v>
+        <v>0.7882</v>
       </c>
       <c r="N3" t="n">
-        <v>0.7265</v>
+        <v>0.876</v>
       </c>
       <c r="O3" t="n">
-        <v>0.7006</v>
+        <v>0.754</v>
       </c>
       <c r="P3" t="n">
-        <v>0.299</v>
+        <v>0.2549</v>
       </c>
     </row>
     <row r="4">
@@ -635,47 +635,47 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.9311910835773167</v>
+        <v>0.952742401153302</v>
       </c>
       <c r="E4" t="n">
-        <v>0.003317252667101671</v>
+        <v>0.001911927986702732</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7870025454862608</v>
+        <v>0.8303908161318067</v>
       </c>
       <c r="G4" t="n">
-        <v>0.005539922661320788</v>
+        <v>0.004960968429522507</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7545675339196789</v>
+        <v>0.8538239701866471</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8226533198809969</v>
+        <v>0.808414387968506</v>
       </c>
       <c r="J4" t="n">
-        <v>9.345000000000001</v>
+        <v>8.996</v>
       </c>
       <c r="K4" t="n">
-        <v>0.923</v>
+        <v>0.9560999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>0.77</v>
+        <v>0.829</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7289</v>
+        <v>0.844</v>
       </c>
       <c r="N4" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.8144</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6671</v>
+        <v>0.76</v>
       </c>
       <c r="P4" t="n">
-        <v>0.3356</v>
+        <v>0.2365</v>
       </c>
     </row>
     <row r="5">
@@ -691,58 +691,58 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.9308911136203069</v>
+        <v>0.9521450064881061</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002936380163272879</v>
+        <v>0.001421577006580887</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7855424675554907</v>
+        <v>0.8275310690545604</v>
       </c>
       <c r="G5" t="n">
-        <v>0.002488758031695132</v>
+        <v>0.005032620104307153</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7465867680398576</v>
+        <v>0.8694951037985138</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8290104374082657</v>
+        <v>0.7896000730238919</v>
       </c>
       <c r="J5" t="n">
-        <v>14.293</v>
+        <v>25.148</v>
       </c>
       <c r="K5" t="n">
-        <v>0.9261</v>
+        <v>0.9564</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7725</v>
+        <v>0.8334</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7282</v>
+        <v>0.8641</v>
       </c>
       <c r="N5" t="n">
-        <v>0.8226</v>
+        <v>0.8048</v>
       </c>
       <c r="O5" t="n">
-        <v>0.6701</v>
+        <v>0.7679</v>
       </c>
       <c r="P5" t="n">
-        <v>0.3337</v>
+        <v>0.2357</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Stacking</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -751,211 +751,211 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.9307603492573528</v>
+        <v>0.9519103293169776</v>
       </c>
       <c r="E6" t="n">
-        <v>0.003369638422393489</v>
+        <v>0.001557221927747491</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7881854927351709</v>
+        <v>0.8243113937095341</v>
       </c>
       <c r="G6" t="n">
-        <v>0.006441266113322218</v>
+        <v>0.00332940937553879</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8306076336509782</v>
+        <v>0.7834979572897383</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7501884161812543</v>
+        <v>0.8696920960522669</v>
       </c>
       <c r="J6" t="n">
-        <v>1503.055</v>
+        <v>16.487</v>
       </c>
       <c r="K6" t="n">
-        <v>0.9358</v>
+        <v>0.9567</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7988</v>
+        <v>0.8244</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8356</v>
+        <v>0.7766</v>
       </c>
       <c r="N6" t="n">
-        <v>0.7651</v>
+        <v>0.8784999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.7208</v>
+        <v>0.7454</v>
       </c>
       <c r="P6" t="n">
-        <v>0.2855</v>
+        <v>0.2621</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Stacking</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.9307603492573528</v>
+        <v>0.9511099837908592</v>
       </c>
       <c r="E7" t="n">
-        <v>0.003369638422393489</v>
+        <v>0.001457607870015335</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7881854927351709</v>
+        <v>0.8271588510229348</v>
       </c>
       <c r="G7" t="n">
-        <v>0.006441266113322218</v>
+        <v>0.00510875703307486</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8306076336509782</v>
+        <v>0.8482930033478343</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7501884161812543</v>
+        <v>0.8072708047410601</v>
       </c>
       <c r="J7" t="n">
-        <v>1883.698</v>
+        <v>19.148</v>
       </c>
       <c r="K7" t="n">
-        <v>0.9358</v>
+        <v>0.9550999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7988</v>
+        <v>0.8279</v>
       </c>
       <c r="M7" t="n">
-        <v>0.8356</v>
+        <v>0.8418</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7651</v>
+        <v>0.8144</v>
       </c>
       <c r="O7" t="n">
-        <v>0.7208</v>
+        <v>0.7584</v>
       </c>
       <c r="P7" t="n">
-        <v>0.2855</v>
+        <v>0.241</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Stacking</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.9301020627141068</v>
+        <v>0.9509454529582371</v>
       </c>
       <c r="E8" t="n">
-        <v>0.003615020362795819</v>
+        <v>0.002072358484271208</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7912076238273901</v>
+        <v>0.8251813955488357</v>
       </c>
       <c r="G8" t="n">
-        <v>0.004430685515000163</v>
+        <v>0.004311349696083499</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8233056141907756</v>
+        <v>0.8560836957613203</v>
       </c>
       <c r="I8" t="n">
-        <v>0.761759391122912</v>
+        <v>0.7965917875586352</v>
       </c>
       <c r="J8" t="n">
-        <v>10.57</v>
+        <v>1442.575</v>
       </c>
       <c r="K8" t="n">
-        <v>0.9222</v>
+        <v>0.9535</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7691</v>
+        <v>0.8273</v>
       </c>
       <c r="M8" t="n">
-        <v>0.762</v>
+        <v>0.8483000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>0.7763</v>
+        <v>0.8073</v>
       </c>
       <c r="O8" t="n">
-        <v>0.6723</v>
+        <v>0.7584</v>
       </c>
       <c r="P8" t="n">
-        <v>0.3156</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>Stacking</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.9295569988554219</v>
+        <v>0.9509454529582371</v>
       </c>
       <c r="E9" t="n">
-        <v>0.003125262472040333</v>
+        <v>0.002072358484271208</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7855041140985022</v>
+        <v>0.8251813955488357</v>
       </c>
       <c r="G9" t="n">
-        <v>0.002663098842694002</v>
+        <v>0.004311349696083499</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8201749687954146</v>
+        <v>0.8560836957613203</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7538773344017654</v>
+        <v>0.7965917875586352</v>
       </c>
       <c r="J9" t="n">
-        <v>19.323</v>
+        <v>1390.184</v>
       </c>
       <c r="K9" t="n">
-        <v>0.9242</v>
+        <v>0.9535</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7788</v>
+        <v>0.8273</v>
       </c>
       <c r="M9" t="n">
-        <v>0.7798</v>
+        <v>0.8483000000000001</v>
       </c>
       <c r="N9" t="n">
-        <v>0.7778</v>
+        <v>0.8073</v>
       </c>
       <c r="O9" t="n">
-        <v>0.6876</v>
+        <v>0.7584</v>
       </c>
       <c r="P9" t="n">
-        <v>0.3116</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="10">
@@ -971,103 +971,103 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.9291247191504812</v>
+        <v>0.9496473590790206</v>
       </c>
       <c r="E10" t="n">
-        <v>0.003320779901018898</v>
+        <v>0.001591566008043649</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7811163067495628</v>
+        <v>0.8223499537643276</v>
       </c>
       <c r="G10" t="n">
-        <v>0.006795949429838209</v>
+        <v>0.00331651332297705</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8527291742676015</v>
+        <v>0.7822586669537891</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7209492944389559</v>
+        <v>0.8668948124764227</v>
       </c>
       <c r="J10" t="n">
-        <v>21.669</v>
+        <v>34.533</v>
       </c>
       <c r="K10" t="n">
-        <v>0.9255</v>
+        <v>0.953</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7766</v>
+        <v>0.8188</v>
       </c>
       <c r="M10" t="n">
-        <v>0.8401999999999999</v>
+        <v>0.7702</v>
       </c>
       <c r="N10" t="n">
-        <v>0.7219</v>
+        <v>0.8739</v>
       </c>
       <c r="O10" t="n">
-        <v>0.6938</v>
+        <v>0.737</v>
       </c>
       <c r="P10" t="n">
-        <v>0.2979</v>
+        <v>0.2746</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Stacking</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.9291065767684914</v>
+        <v>0.9495410566153544</v>
       </c>
       <c r="E11" t="n">
-        <v>0.003556340034782772</v>
+        <v>0.001841139854607562</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7878604723957467</v>
+        <v>0.8218303735581662</v>
       </c>
       <c r="G11" t="n">
-        <v>0.005884427512063179</v>
+        <v>0.005615591251413946</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7810071136288008</v>
+        <v>0.8744512182239209</v>
       </c>
       <c r="I11" t="n">
-        <v>0.7950660405783427</v>
+        <v>0.7753606564395522</v>
       </c>
       <c r="J11" t="n">
-        <v>3609.714</v>
+        <v>27.511</v>
       </c>
       <c r="K11" t="n">
-        <v>0.9339</v>
+        <v>0.9536</v>
       </c>
       <c r="L11" t="n">
-        <v>0.7965</v>
+        <v>0.8274</v>
       </c>
       <c r="M11" t="n">
-        <v>0.7798</v>
+        <v>0.8691</v>
       </c>
       <c r="N11" t="n">
-        <v>0.8139</v>
+        <v>0.7895</v>
       </c>
       <c r="O11" t="n">
-        <v>0.7098</v>
+        <v>0.7608</v>
       </c>
       <c r="P11" t="n">
-        <v>0.3021</v>
+        <v>0.2425</v>
       </c>
     </row>
     <row r="12">
@@ -1083,58 +1083,58 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.9286477102997148</v>
+        <v>0.9492213590114341</v>
       </c>
       <c r="E12" t="n">
-        <v>0.003302395485081426</v>
+        <v>0.001707534404035993</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7847601758073608</v>
+        <v>0.8234345236250021</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006420774015971335</v>
+        <v>0.004391626251727939</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7438051311286004</v>
+        <v>0.8459320523351781</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8306625221838344</v>
+        <v>0.8023123693910341</v>
       </c>
       <c r="J12" t="n">
-        <v>21.118</v>
+        <v>47.524</v>
       </c>
       <c r="K12" t="n">
-        <v>0.923</v>
+        <v>0.9519</v>
       </c>
       <c r="L12" t="n">
-        <v>0.7747000000000001</v>
+        <v>0.8244</v>
       </c>
       <c r="M12" t="n">
-        <v>0.7429</v>
+        <v>0.8389</v>
       </c>
       <c r="N12" t="n">
-        <v>0.8094</v>
+        <v>0.8104</v>
       </c>
       <c r="O12" t="n">
-        <v>0.6758</v>
+        <v>0.7536</v>
       </c>
       <c r="P12" t="n">
-        <v>0.3261</v>
+        <v>0.2501</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>Stacking</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1143,43 +1143,43 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.9277165208629947</v>
+        <v>0.9488747938285949</v>
       </c>
       <c r="E13" t="n">
-        <v>0.004115470851487426</v>
+        <v>0.002773654872964864</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7857817865369323</v>
+        <v>0.8231545772598434</v>
       </c>
       <c r="G13" t="n">
-        <v>0.006122454155172192</v>
+        <v>0.005135717713261351</v>
       </c>
       <c r="H13" t="n">
-        <v>0.8165921484640132</v>
+        <v>0.8153806817385323</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7574357143376436</v>
+        <v>0.8312981693136481</v>
       </c>
       <c r="J13" t="n">
-        <v>18.515</v>
+        <v>6342.906</v>
       </c>
       <c r="K13" t="n">
-        <v>0.9233</v>
+        <v>0.9514</v>
       </c>
       <c r="L13" t="n">
-        <v>0.7742</v>
+        <v>0.8196</v>
       </c>
       <c r="M13" t="n">
-        <v>0.7788</v>
+        <v>0.7985</v>
       </c>
       <c r="N13" t="n">
-        <v>0.7697000000000001</v>
+        <v>0.8419</v>
       </c>
       <c r="O13" t="n">
-        <v>0.6817</v>
+        <v>0.7422</v>
       </c>
       <c r="P13" t="n">
-        <v>0.308</v>
+        <v>0.262</v>
       </c>
     </row>
     <row r="14">
@@ -1195,114 +1195,114 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.9255995216415347</v>
+        <v>0.9472837262589477</v>
       </c>
       <c r="E14" t="n">
-        <v>0.003787021573586583</v>
+        <v>0.002751049853717754</v>
       </c>
       <c r="F14" t="n">
-        <v>0.7580137134565823</v>
+        <v>0.8169909203107798</v>
       </c>
       <c r="G14" t="n">
-        <v>0.005482087979962167</v>
+        <v>0.00403007160636598</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8572283564913865</v>
+        <v>0.8060355566987134</v>
       </c>
       <c r="I14" t="n">
-        <v>0.6796328772301973</v>
+        <v>0.8285014511882942</v>
       </c>
       <c r="J14" t="n">
-        <v>36.396</v>
+        <v>78.515</v>
       </c>
       <c r="K14" t="n">
-        <v>0.9308</v>
+        <v>0.95</v>
       </c>
       <c r="L14" t="n">
-        <v>0.7693</v>
+        <v>0.8174</v>
       </c>
       <c r="M14" t="n">
-        <v>0.8537</v>
+        <v>0.7942</v>
       </c>
       <c r="N14" t="n">
-        <v>0.7000999999999999</v>
+        <v>0.8419</v>
       </c>
       <c r="O14" t="n">
-        <v>0.6867</v>
+        <v>0.7387</v>
       </c>
       <c r="P14" t="n">
-        <v>0.3002</v>
+        <v>0.2706</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.9254691575849276</v>
+        <v>0.9468460134581385</v>
       </c>
       <c r="E15" t="n">
-        <v>0.003646481622075709</v>
+        <v>0.003213222126478196</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7672089609104129</v>
+        <v>0.8119230545151636</v>
       </c>
       <c r="G15" t="n">
-        <v>0.004973036242139429</v>
+        <v>0.003672167353116909</v>
       </c>
       <c r="H15" t="n">
-        <v>0.8432462746004135</v>
+        <v>0.8745186228742853</v>
       </c>
       <c r="I15" t="n">
-        <v>0.7040407092041608</v>
+        <v>0.7579444582216905</v>
       </c>
       <c r="J15" t="n">
-        <v>39.122</v>
+        <v>22.354</v>
       </c>
       <c r="K15" t="n">
-        <v>0.9199000000000001</v>
+        <v>0.9500999999999999</v>
       </c>
       <c r="L15" t="n">
-        <v>0.774</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="M15" t="n">
-        <v>0.8489</v>
+        <v>0.8622</v>
       </c>
       <c r="N15" t="n">
-        <v>0.7112000000000001</v>
+        <v>0.7728</v>
       </c>
       <c r="O15" t="n">
-        <v>0.6918</v>
+        <v>0.7443</v>
       </c>
       <c r="P15" t="n">
-        <v>0.3064</v>
+        <v>0.2576</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>MLP + EBM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>MLP</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1311,54 +1311,54 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.9254691575849276</v>
+        <v>0.9464621706301779</v>
       </c>
       <c r="E16" t="n">
-        <v>0.003646481622075709</v>
+        <v>0.002383645514213897</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7672089609104129</v>
+        <v>0.813205080862484</v>
       </c>
       <c r="G16" t="n">
-        <v>0.004973036242139429</v>
+        <v>0.002406446270486991</v>
       </c>
       <c r="H16" t="n">
-        <v>0.8432462746004135</v>
+        <v>0.8772146191398633</v>
       </c>
       <c r="I16" t="n">
-        <v>0.7040407092041608</v>
+        <v>0.7585815593670509</v>
       </c>
       <c r="J16" t="n">
-        <v>32.026</v>
+        <v>6.195</v>
       </c>
       <c r="K16" t="n">
-        <v>0.9199000000000001</v>
+        <v>0.9530999999999999</v>
       </c>
       <c r="L16" t="n">
-        <v>0.774</v>
+        <v>0.8310999999999999</v>
       </c>
       <c r="M16" t="n">
-        <v>0.8489</v>
+        <v>0.8512999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>0.7112000000000001</v>
+        <v>0.8119</v>
       </c>
       <c r="O16" t="n">
-        <v>0.6918</v>
+        <v>0.7635999999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>0.3064</v>
+        <v>0.2423</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>MLP + EBM</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Voting</t>
+          <t>MLP</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1367,155 +1367,155 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.9253609085385284</v>
+        <v>0.9464621706301779</v>
       </c>
       <c r="E17" t="n">
-        <v>0.00382201184570054</v>
+        <v>0.002383645514213897</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7780450447876784</v>
+        <v>0.813205080862484</v>
       </c>
       <c r="G17" t="n">
-        <v>0.004658825352115823</v>
+        <v>0.002406446270486991</v>
       </c>
       <c r="H17" t="n">
-        <v>0.817508047908289</v>
+        <v>0.8772146191398633</v>
       </c>
       <c r="I17" t="n">
-        <v>0.742434555164138</v>
+        <v>0.7585815593670509</v>
       </c>
       <c r="J17" t="n">
-        <v>513.6319999999999</v>
+        <v>6.972</v>
       </c>
       <c r="K17" t="n">
-        <v>0.9304</v>
+        <v>0.9530999999999999</v>
       </c>
       <c r="L17" t="n">
-        <v>0.7867</v>
+        <v>0.8310999999999999</v>
       </c>
       <c r="M17" t="n">
-        <v>0.8159</v>
+        <v>0.8512999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>0.7595</v>
+        <v>0.8119</v>
       </c>
       <c r="O17" t="n">
-        <v>0.703</v>
+        <v>0.7635999999999999</v>
       </c>
       <c r="P17" t="n">
-        <v>0.2995</v>
+        <v>0.2423</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Voting</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.9253609085385284</v>
+        <v>0.9463225401639883</v>
       </c>
       <c r="E18" t="n">
-        <v>0.00382201184570054</v>
+        <v>0.002890365512650833</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7780450447876784</v>
+        <v>0.8120138369716026</v>
       </c>
       <c r="G18" t="n">
-        <v>0.004658825352115823</v>
+        <v>0.006330304171625894</v>
       </c>
       <c r="H18" t="n">
-        <v>0.817508047908289</v>
+        <v>0.7843580412773777</v>
       </c>
       <c r="I18" t="n">
-        <v>0.742434555164138</v>
+        <v>0.841849879357099</v>
       </c>
       <c r="J18" t="n">
-        <v>390.557</v>
+        <v>14.862</v>
       </c>
       <c r="K18" t="n">
-        <v>0.9304</v>
+        <v>0.9497</v>
       </c>
       <c r="L18" t="n">
-        <v>0.7867</v>
+        <v>0.8159</v>
       </c>
       <c r="M18" t="n">
-        <v>0.8159</v>
+        <v>0.7775</v>
       </c>
       <c r="N18" t="n">
-        <v>0.7595</v>
+        <v>0.8582</v>
       </c>
       <c r="O18" t="n">
-        <v>0.703</v>
+        <v>0.7343</v>
       </c>
       <c r="P18" t="n">
-        <v>0.2995</v>
+        <v>0.2805</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>Voting</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.9250778506279677</v>
+        <v>0.9449883476342735</v>
       </c>
       <c r="E19" t="n">
-        <v>0.003443392487008852</v>
+        <v>0.002471744951359491</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7787225159442722</v>
+        <v>0.8158304750648921</v>
       </c>
       <c r="G19" t="n">
-        <v>0.005997512743632617</v>
+        <v>0.003505436513881685</v>
       </c>
       <c r="H19" t="n">
-        <v>0.7592287863582301</v>
+        <v>0.8422739919119419</v>
       </c>
       <c r="I19" t="n">
-        <v>0.7993887480199137</v>
+        <v>0.7912527232499509</v>
       </c>
       <c r="J19" t="n">
-        <v>16.146</v>
+        <v>656.528</v>
       </c>
       <c r="K19" t="n">
-        <v>0.9296</v>
+        <v>0.9483</v>
       </c>
       <c r="L19" t="n">
-        <v>0.7851</v>
+        <v>0.8176</v>
       </c>
       <c r="M19" t="n">
-        <v>0.7522</v>
+        <v>0.8313</v>
       </c>
       <c r="N19" t="n">
-        <v>0.821</v>
+        <v>0.8043</v>
       </c>
       <c r="O19" t="n">
-        <v>0.6907</v>
+        <v>0.7439</v>
       </c>
       <c r="P19" t="n">
-        <v>0.3284</v>
+        <v>0.2636</v>
       </c>
     </row>
     <row r="20">
@@ -1531,58 +1531,58 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.924575927827392</v>
+        <v>0.9449883476342735</v>
       </c>
       <c r="E20" t="n">
-        <v>0.00403692349496118</v>
+        <v>0.002471744951359491</v>
       </c>
       <c r="F20" t="n">
-        <v>0.7841880159374434</v>
+        <v>0.8158304750648921</v>
       </c>
       <c r="G20" t="n">
-        <v>0.006443181769639867</v>
+        <v>0.003505436513881685</v>
       </c>
       <c r="H20" t="n">
-        <v>0.786120607203334</v>
+        <v>0.8422739919119419</v>
       </c>
       <c r="I20" t="n">
-        <v>0.7824804858996843</v>
+        <v>0.7912527232499509</v>
       </c>
       <c r="J20" t="n">
-        <v>1877.52</v>
+        <v>481.012</v>
       </c>
       <c r="K20" t="n">
-        <v>0.9296</v>
+        <v>0.9483</v>
       </c>
       <c r="L20" t="n">
-        <v>0.7889</v>
+        <v>0.8176</v>
       </c>
       <c r="M20" t="n">
-        <v>0.7783</v>
+        <v>0.8313</v>
       </c>
       <c r="N20" t="n">
-        <v>0.7997</v>
+        <v>0.8043</v>
       </c>
       <c r="O20" t="n">
-        <v>0.6999</v>
+        <v>0.7439</v>
       </c>
       <c r="P20" t="n">
-        <v>0.3085</v>
+        <v>0.2636</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>Voting</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1591,43 +1591,43 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.9240604004900707</v>
+        <v>0.944761622362701</v>
       </c>
       <c r="E21" t="n">
-        <v>0.003663125512128296</v>
+        <v>0.002644847308576271</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7782213124346666</v>
+        <v>0.8200644394623776</v>
       </c>
       <c r="G21" t="n">
-        <v>0.006809658645278932</v>
+        <v>0.004151467032299099</v>
       </c>
       <c r="H21" t="n">
-        <v>0.7740562378479641</v>
+        <v>0.8147946097158089</v>
       </c>
       <c r="I21" t="n">
-        <v>0.7826072275881678</v>
+        <v>0.8257047330629403</v>
       </c>
       <c r="J21" t="n">
-        <v>15.915</v>
+        <v>1731.173</v>
       </c>
       <c r="K21" t="n">
-        <v>0.9288</v>
+        <v>0.9481000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>0.7831</v>
+        <v>0.8236</v>
       </c>
       <c r="M21" t="n">
-        <v>0.7675999999999999</v>
+        <v>0.8088</v>
       </c>
       <c r="N21" t="n">
-        <v>0.7992</v>
+        <v>0.8388</v>
       </c>
       <c r="O21" t="n">
-        <v>0.6908</v>
+        <v>0.7487</v>
       </c>
       <c r="P21" t="n">
-        <v>0.3168</v>
+        <v>0.2711</v>
       </c>
     </row>
     <row r="22">
@@ -1643,58 +1643,58 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.9222753475760725</v>
+        <v>0.9446026324439973</v>
       </c>
       <c r="E22" t="n">
-        <v>0.004139844727486687</v>
+        <v>0.002240480118703075</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7693477151049755</v>
+        <v>0.8102563390992875</v>
       </c>
       <c r="G22" t="n">
-        <v>0.004717766394153992</v>
+        <v>0.005350022911762434</v>
       </c>
       <c r="H22" t="n">
-        <v>0.7834716267548076</v>
+        <v>0.8581033800328084</v>
       </c>
       <c r="I22" t="n">
-        <v>0.7559101289146339</v>
+        <v>0.7677332139963536</v>
       </c>
       <c r="J22" t="n">
-        <v>68.5</v>
+        <v>26.029</v>
       </c>
       <c r="K22" t="n">
-        <v>0.9195</v>
+        <v>0.9489</v>
       </c>
       <c r="L22" t="n">
-        <v>0.7702</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="M22" t="n">
-        <v>0.7754</v>
+        <v>0.8514</v>
       </c>
       <c r="N22" t="n">
-        <v>0.7651</v>
+        <v>0.7834</v>
       </c>
       <c r="O22" t="n">
-        <v>0.6761</v>
+        <v>0.7443</v>
       </c>
       <c r="P22" t="n">
-        <v>0.3142</v>
+        <v>0.2563</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MLP + EBM</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EBM</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1703,99 +1703,99 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.9202268779529679</v>
+        <v>0.9446026324439973</v>
       </c>
       <c r="E23" t="n">
-        <v>0.003602000107884734</v>
+        <v>0.002240480118703075</v>
       </c>
       <c r="F23" t="n">
-        <v>0.7671836754230297</v>
+        <v>0.8102563390992875</v>
       </c>
       <c r="G23" t="n">
-        <v>0.007072489870372478</v>
+        <v>0.005350022911762434</v>
       </c>
       <c r="H23" t="n">
-        <v>0.8340643750835186</v>
+        <v>0.8581033800328084</v>
       </c>
       <c r="I23" t="n">
-        <v>0.7105242453053473</v>
+        <v>0.7677332139963536</v>
       </c>
       <c r="J23" t="n">
-        <v>263.372</v>
+        <v>42.487</v>
       </c>
       <c r="K23" t="n">
-        <v>0.9255</v>
+        <v>0.9489</v>
       </c>
       <c r="L23" t="n">
-        <v>0.7719</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>0.8354</v>
+        <v>0.8514</v>
       </c>
       <c r="N23" t="n">
-        <v>0.7173</v>
+        <v>0.7834</v>
       </c>
       <c r="O23" t="n">
-        <v>0.6874</v>
+        <v>0.7443</v>
       </c>
       <c r="P23" t="n">
-        <v>0.2971</v>
+        <v>0.2563</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MLP + EBM</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EBM</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.9202268779529679</v>
+        <v>0.9433683738755994</v>
       </c>
       <c r="E24" t="n">
-        <v>0.003602000107884734</v>
+        <v>0.002063542596344094</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7671836754230297</v>
+        <v>0.813106416063533</v>
       </c>
       <c r="G24" t="n">
-        <v>0.007072489870372478</v>
+        <v>0.003923118116496006</v>
       </c>
       <c r="H24" t="n">
-        <v>0.8340643750835186</v>
+        <v>0.8158289994304611</v>
       </c>
       <c r="I24" t="n">
-        <v>0.7105242453053473</v>
+        <v>0.8105763475291026</v>
       </c>
       <c r="J24" t="n">
-        <v>265.606</v>
+        <v>73.32599999999999</v>
       </c>
       <c r="K24" t="n">
-        <v>0.9255</v>
+        <v>0.947</v>
       </c>
       <c r="L24" t="n">
-        <v>0.7719</v>
+        <v>0.8163</v>
       </c>
       <c r="M24" t="n">
-        <v>0.8354</v>
+        <v>0.8048</v>
       </c>
       <c r="N24" t="n">
-        <v>0.7173</v>
+        <v>0.8282</v>
       </c>
       <c r="O24" t="n">
-        <v>0.6874</v>
+        <v>0.7389</v>
       </c>
       <c r="P24" t="n">
-        <v>0.2971</v>
+        <v>0.2687</v>
       </c>
     </row>
     <row r="25">
@@ -1815,43 +1815,43 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.9195671996866903</v>
+        <v>0.9379721344826782</v>
       </c>
       <c r="E25" t="n">
-        <v>0.004724682936439577</v>
+        <v>0.003904515896731891</v>
       </c>
       <c r="F25" t="n">
-        <v>0.7742913987501752</v>
+        <v>0.8087287022616166</v>
       </c>
       <c r="G25" t="n">
-        <v>0.005569902515071754</v>
+        <v>0.004188423177670716</v>
       </c>
       <c r="H25" t="n">
-        <v>0.8145387034019862</v>
+        <v>0.8398505034006488</v>
       </c>
       <c r="I25" t="n">
-        <v>0.7381117669439259</v>
+        <v>0.7800661738631012</v>
       </c>
       <c r="J25" t="n">
-        <v>840.438</v>
+        <v>1777.304</v>
       </c>
       <c r="K25" t="n">
-        <v>0.9243</v>
+        <v>0.9422</v>
       </c>
       <c r="L25" t="n">
-        <v>0.783</v>
+        <v>0.8099</v>
       </c>
       <c r="M25" t="n">
-        <v>0.8167</v>
+        <v>0.8349</v>
       </c>
       <c r="N25" t="n">
-        <v>0.7519</v>
+        <v>0.7865</v>
       </c>
       <c r="O25" t="n">
-        <v>0.6984</v>
+        <v>0.7347</v>
       </c>
       <c r="P25" t="n">
-        <v>0.3022</v>
+        <v>0.2665</v>
       </c>
     </row>
     <row r="26">
@@ -1867,47 +1867,47 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.9184766557449542</v>
+        <v>0.937399108755538</v>
       </c>
       <c r="E26" t="n">
-        <v>0.004254839454904571</v>
+        <v>0.005060147566467056</v>
       </c>
       <c r="F26" t="n">
-        <v>0.7638435817419618</v>
+        <v>0.807845391480854</v>
       </c>
       <c r="G26" t="n">
-        <v>0.007048004886076593</v>
+        <v>0.01031190045657124</v>
       </c>
       <c r="H26" t="n">
-        <v>0.8163151563330622</v>
+        <v>0.7955793945456492</v>
       </c>
       <c r="I26" t="n">
-        <v>0.7181532225427338</v>
+        <v>0.8206202022535625</v>
       </c>
       <c r="J26" t="n">
-        <v>14.569</v>
+        <v>19.323</v>
       </c>
       <c r="K26" t="n">
-        <v>0.9262</v>
+        <v>0.9465</v>
       </c>
       <c r="L26" t="n">
-        <v>0.7708</v>
+        <v>0.8193</v>
       </c>
       <c r="M26" t="n">
-        <v>0.8329</v>
+        <v>0.7984</v>
       </c>
       <c r="N26" t="n">
-        <v>0.7173</v>
+        <v>0.8414</v>
       </c>
       <c r="O26" t="n">
-        <v>0.6858</v>
+        <v>0.7418</v>
       </c>
       <c r="P26" t="n">
-        <v>0.2978</v>
+        <v>0.2923</v>
       </c>
     </row>
     <row r="27">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>EBM</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1927,43 +1927,43 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.9184766557449542</v>
+        <v>0.9373762069707006</v>
       </c>
       <c r="E27" t="n">
-        <v>0.004254839454904571</v>
+        <v>0.002621040993716543</v>
       </c>
       <c r="F27" t="n">
-        <v>0.7638435817419618</v>
+        <v>0.8009504015452423</v>
       </c>
       <c r="G27" t="n">
-        <v>0.007048004886076593</v>
+        <v>0.005202682637965449</v>
       </c>
       <c r="H27" t="n">
-        <v>0.8163151563330622</v>
+        <v>0.8503856976864406</v>
       </c>
       <c r="I27" t="n">
-        <v>0.7181532225427338</v>
+        <v>0.7571827964111664</v>
       </c>
       <c r="J27" t="n">
-        <v>14.312</v>
+        <v>428.258</v>
       </c>
       <c r="K27" t="n">
-        <v>0.9262</v>
+        <v>0.9421</v>
       </c>
       <c r="L27" t="n">
-        <v>0.7708</v>
+        <v>0.8071</v>
       </c>
       <c r="M27" t="n">
-        <v>0.8329</v>
+        <v>0.8478</v>
       </c>
       <c r="N27" t="n">
-        <v>0.7173</v>
+        <v>0.7702</v>
       </c>
       <c r="O27" t="n">
-        <v>0.6858</v>
+        <v>0.7327</v>
       </c>
       <c r="P27" t="n">
-        <v>0.2978</v>
+        <v>0.2654</v>
       </c>
     </row>
     <row r="28">
@@ -1974,119 +1974,119 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>EBM</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.9096239909896064</v>
+        <v>0.9373762069707006</v>
       </c>
       <c r="E28" t="n">
-        <v>0.002737100653331916</v>
+        <v>0.002621040993716543</v>
       </c>
       <c r="F28" t="n">
-        <v>0.7572306532482551</v>
+        <v>0.8009504015452423</v>
       </c>
       <c r="G28" t="n">
-        <v>0.008394077963791647</v>
+        <v>0.005202682637965449</v>
       </c>
       <c r="H28" t="n">
-        <v>0.7224095083836887</v>
+        <v>0.8503856976864406</v>
       </c>
       <c r="I28" t="n">
-        <v>0.7967202255985899</v>
+        <v>0.7571827964111664</v>
       </c>
       <c r="J28" t="n">
-        <v>30.771</v>
+        <v>280.69</v>
       </c>
       <c r="K28" t="n">
-        <v>0.9187</v>
+        <v>0.9421</v>
       </c>
       <c r="L28" t="n">
-        <v>0.7713</v>
+        <v>0.8071</v>
       </c>
       <c r="M28" t="n">
-        <v>0.7354000000000001</v>
+        <v>0.8478</v>
       </c>
       <c r="N28" t="n">
-        <v>0.8109</v>
+        <v>0.7702</v>
       </c>
       <c r="O28" t="n">
-        <v>0.6701</v>
+        <v>0.7327</v>
       </c>
       <c r="P28" t="n">
-        <v>0.3719</v>
+        <v>0.2654</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.9088978328670831</v>
+        <v>0.9315129619923168</v>
       </c>
       <c r="E29" t="n">
-        <v>0.005891850327644642</v>
+        <v>0.00376073451208329</v>
       </c>
       <c r="F29" t="n">
-        <v>0.7484429778343922</v>
+        <v>0.7591554666450639</v>
       </c>
       <c r="G29" t="n">
-        <v>0.007045173669809596</v>
+        <v>0.006986982179453731</v>
       </c>
       <c r="H29" t="n">
-        <v>0.7184990455026184</v>
+        <v>0.8768327532554583</v>
       </c>
       <c r="I29" t="n">
-        <v>0.7810824499515732</v>
+        <v>0.6695891840630204</v>
       </c>
       <c r="J29" t="n">
-        <v>31.037</v>
+        <v>35.522</v>
       </c>
       <c r="K29" t="n">
-        <v>0.9133</v>
+        <v>0.9336</v>
       </c>
       <c r="L29" t="n">
-        <v>0.7551</v>
+        <v>0.761</v>
       </c>
       <c r="M29" t="n">
-        <v>0.7111</v>
+        <v>0.8643</v>
       </c>
       <c r="N29" t="n">
-        <v>0.8048</v>
+        <v>0.6797</v>
       </c>
       <c r="O29" t="n">
-        <v>0.6447000000000001</v>
+        <v>0.678</v>
       </c>
       <c r="P29" t="n">
-        <v>0.4631</v>
+        <v>0.3122</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2095,155 +2095,155 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.9073468196712163</v>
+        <v>0.9313679768742575</v>
       </c>
       <c r="E30" t="n">
-        <v>0.005419817326884455</v>
+        <v>0.003516553961544682</v>
       </c>
       <c r="F30" t="n">
-        <v>0.7346021919440012</v>
+        <v>0.7810657033018569</v>
       </c>
       <c r="G30" t="n">
-        <v>0.008623850829764327</v>
+        <v>0.007559627176103657</v>
       </c>
       <c r="H30" t="n">
-        <v>0.8117269994874123</v>
+        <v>0.7330423223469913</v>
       </c>
       <c r="I30" t="n">
-        <v>0.6712423189609281</v>
+        <v>0.836002959729424</v>
       </c>
       <c r="J30" t="n">
-        <v>18.325</v>
+        <v>2.793</v>
       </c>
       <c r="K30" t="n">
-        <v>0.9117</v>
+        <v>0.9343</v>
       </c>
       <c r="L30" t="n">
-        <v>0.7396</v>
+        <v>0.7828000000000001</v>
       </c>
       <c r="M30" t="n">
-        <v>0.8075</v>
+        <v>0.7221</v>
       </c>
       <c r="N30" t="n">
-        <v>0.6823</v>
+        <v>0.8546</v>
       </c>
       <c r="O30" t="n">
-        <v>0.6443</v>
+        <v>0.6819</v>
       </c>
       <c r="P30" t="n">
-        <v>0.4205</v>
+        <v>0.3506</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.9073468196712163</v>
+        <v>0.9308044637766206</v>
       </c>
       <c r="E31" t="n">
-        <v>0.005419817326884455</v>
+        <v>0.003272936094553819</v>
       </c>
       <c r="F31" t="n">
-        <v>0.7346021919440012</v>
+        <v>0.783444623490177</v>
       </c>
       <c r="G31" t="n">
-        <v>0.008623850829764327</v>
+        <v>0.009242881824032642</v>
       </c>
       <c r="H31" t="n">
-        <v>0.8117269994874123</v>
+        <v>0.7465855429302748</v>
       </c>
       <c r="I31" t="n">
-        <v>0.6712423189609281</v>
+        <v>0.8243067778934707</v>
       </c>
       <c r="J31" t="n">
-        <v>19.987</v>
+        <v>34.249</v>
       </c>
       <c r="K31" t="n">
-        <v>0.9117</v>
+        <v>0.9332</v>
       </c>
       <c r="L31" t="n">
-        <v>0.7396</v>
+        <v>0.785</v>
       </c>
       <c r="M31" t="n">
-        <v>0.8075</v>
+        <v>0.7346</v>
       </c>
       <c r="N31" t="n">
-        <v>0.6823</v>
+        <v>0.8429</v>
       </c>
       <c r="O31" t="n">
-        <v>0.6443</v>
+        <v>0.6873</v>
       </c>
       <c r="P31" t="n">
-        <v>0.4205</v>
+        <v>0.3451</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.9064751028619534</v>
+        <v>0.9298593588287318</v>
       </c>
       <c r="E32" t="n">
-        <v>0.004133827840274739</v>
+        <v>0.002940966150935203</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7449095387311913</v>
+        <v>0.7857642160266411</v>
       </c>
       <c r="G32" t="n">
-        <v>0.007181450334187754</v>
+        <v>0.007518361017691409</v>
       </c>
       <c r="H32" t="n">
-        <v>0.7081655179884478</v>
+        <v>0.7545141466774683</v>
       </c>
       <c r="I32" t="n">
-        <v>0.7859125280402859</v>
+        <v>0.8201101659112517</v>
       </c>
       <c r="J32" t="n">
-        <v>7.072</v>
+        <v>71.434</v>
       </c>
       <c r="K32" t="n">
-        <v>0.913</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="L32" t="n">
-        <v>0.7564</v>
+        <v>0.7861</v>
       </c>
       <c r="M32" t="n">
-        <v>0.7065</v>
+        <v>0.7417</v>
       </c>
       <c r="N32" t="n">
-        <v>0.8139</v>
+        <v>0.8363</v>
       </c>
       <c r="O32" t="n">
-        <v>0.6454</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P32" t="n">
-        <v>0.4136</v>
+        <v>0.445</v>
       </c>
     </row>
     <row r="33">
@@ -2263,43 +2263,43 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.9062719112250728</v>
+        <v>0.9282010462024315</v>
       </c>
       <c r="E33" t="n">
-        <v>0.003155251030847576</v>
+        <v>0.003252072683053184</v>
       </c>
       <c r="F33" t="n">
-        <v>0.702128629123305</v>
+        <v>0.7680192654030435</v>
       </c>
       <c r="G33" t="n">
-        <v>0.01701650551630925</v>
+        <v>0.01137668644677119</v>
       </c>
       <c r="H33" t="n">
-        <v>0.8475576441688654</v>
+        <v>0.830378849828832</v>
       </c>
       <c r="I33" t="n">
-        <v>0.6025966294304055</v>
+        <v>0.7151064945219965</v>
       </c>
       <c r="J33" t="n">
-        <v>14.083</v>
+        <v>20.731</v>
       </c>
       <c r="K33" t="n">
-        <v>0.914</v>
+        <v>0.9339</v>
       </c>
       <c r="L33" t="n">
-        <v>0.7071</v>
+        <v>0.7713</v>
       </c>
       <c r="M33" t="n">
-        <v>0.8773</v>
+        <v>0.8138</v>
       </c>
       <c r="N33" t="n">
-        <v>0.5923</v>
+        <v>0.7331</v>
       </c>
       <c r="O33" t="n">
-        <v>0.6168</v>
+        <v>0.6836</v>
       </c>
       <c r="P33" t="n">
-        <v>0.3278</v>
+        <v>0.2924</v>
       </c>
     </row>
     <row r="34">
@@ -2319,334 +2319,334 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.9062719112250728</v>
+        <v>0.9282010462024315</v>
       </c>
       <c r="E34" t="n">
-        <v>0.003155251030847576</v>
+        <v>0.003252072683053184</v>
       </c>
       <c r="F34" t="n">
-        <v>0.702128629123305</v>
+        <v>0.7680192654030435</v>
       </c>
       <c r="G34" t="n">
-        <v>0.01701650551630925</v>
+        <v>0.01137668644677119</v>
       </c>
       <c r="H34" t="n">
-        <v>0.8475576441688654</v>
+        <v>0.830378849828832</v>
       </c>
       <c r="I34" t="n">
-        <v>0.6025966294304055</v>
+        <v>0.7151064945219965</v>
       </c>
       <c r="J34" t="n">
-        <v>6.348</v>
+        <v>18.024</v>
       </c>
       <c r="K34" t="n">
-        <v>0.914</v>
+        <v>0.9339</v>
       </c>
       <c r="L34" t="n">
-        <v>0.7071</v>
+        <v>0.7713</v>
       </c>
       <c r="M34" t="n">
-        <v>0.8773</v>
+        <v>0.8138</v>
       </c>
       <c r="N34" t="n">
-        <v>0.5923</v>
+        <v>0.7331</v>
       </c>
       <c r="O34" t="n">
-        <v>0.6168</v>
+        <v>0.6836</v>
       </c>
       <c r="P34" t="n">
-        <v>0.3278</v>
+        <v>0.2924</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SVM_RBF</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.9055556282596344</v>
+        <v>0.9240837379510936</v>
       </c>
       <c r="E35" t="n">
-        <v>0.003415658412659005</v>
+        <v>0.003312467116935505</v>
       </c>
       <c r="F35" t="n">
-        <v>0.7564983454614655</v>
+        <v>0.7531045823849295</v>
       </c>
       <c r="G35" t="n">
-        <v>0.006123515596986275</v>
+        <v>0.007630946081345134</v>
       </c>
       <c r="H35" t="n">
-        <v>0.7119822164425902</v>
+        <v>0.8313178176975002</v>
       </c>
       <c r="I35" t="n">
-        <v>0.8071431744875202</v>
+        <v>0.6885311292611743</v>
       </c>
       <c r="J35" t="n">
-        <v>112.901</v>
+        <v>31.611</v>
       </c>
       <c r="K35" t="n">
-        <v>0.9142</v>
+        <v>0.9301</v>
       </c>
       <c r="L35" t="n">
-        <v>0.7623</v>
+        <v>0.7606000000000001</v>
       </c>
       <c r="M35" t="n">
-        <v>0.7079</v>
+        <v>0.8269</v>
       </c>
       <c r="N35" t="n">
-        <v>0.8256</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="O35" t="n">
-        <v>0.653</v>
+        <v>0.6724</v>
       </c>
       <c r="P35" t="n">
-        <v>0.3252</v>
+        <v>0.4058</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.9052964237555472</v>
+        <v>0.9240837379510936</v>
       </c>
       <c r="E36" t="n">
-        <v>0.003862990540722517</v>
+        <v>0.003312467116935505</v>
       </c>
       <c r="F36" t="n">
-        <v>0.7441482098143479</v>
+        <v>0.7531045823849295</v>
       </c>
       <c r="G36" t="n">
-        <v>0.007615210426067979</v>
+        <v>0.007630946081345134</v>
       </c>
       <c r="H36" t="n">
-        <v>0.7178071943882411</v>
+        <v>0.8313178176975002</v>
       </c>
       <c r="I36" t="n">
-        <v>0.7726911646745307</v>
+        <v>0.6885311292611743</v>
       </c>
       <c r="J36" t="n">
-        <v>7.963</v>
+        <v>33.396</v>
       </c>
       <c r="K36" t="n">
-        <v>0.9119</v>
+        <v>0.9301</v>
       </c>
       <c r="L36" t="n">
-        <v>0.7532</v>
+        <v>0.7606000000000001</v>
       </c>
       <c r="M36" t="n">
-        <v>0.7155</v>
+        <v>0.8269</v>
       </c>
       <c r="N36" t="n">
-        <v>0.7951</v>
+        <v>0.7040999999999999</v>
       </c>
       <c r="O36" t="n">
-        <v>0.6434</v>
+        <v>0.6724</v>
       </c>
       <c r="P36" t="n">
-        <v>0.4106</v>
+        <v>0.4058</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Ensambles</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
+          <t>Bagging</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.905201441677766</v>
+        <v>0.9239479055348996</v>
       </c>
       <c r="E37" t="n">
-        <v>0.004635262884190471</v>
+        <v>0.001883537286232897</v>
       </c>
       <c r="F37" t="n">
-        <v>0.676398143613919</v>
+        <v>0.7685357021647838</v>
       </c>
       <c r="G37" t="n">
-        <v>0.01150729959634567</v>
+        <v>0.004666734889156638</v>
       </c>
       <c r="H37" t="n">
-        <v>0.8836132567534383</v>
+        <v>0.7118950317075459</v>
       </c>
       <c r="I37" t="n">
-        <v>0.5481809053831694</v>
+        <v>0.8353645661257998</v>
       </c>
       <c r="J37" t="n">
-        <v>6.286</v>
+        <v>35.549</v>
       </c>
       <c r="K37" t="n">
-        <v>0.9129</v>
+        <v>0.93</v>
       </c>
       <c r="L37" t="n">
-        <v>0.6938</v>
+        <v>0.7708</v>
       </c>
       <c r="M37" t="n">
-        <v>0.8804</v>
+        <v>0.7163</v>
       </c>
       <c r="N37" t="n">
-        <v>0.5724</v>
+        <v>0.8343</v>
       </c>
       <c r="O37" t="n">
-        <v>0.6021</v>
+        <v>0.6655</v>
       </c>
       <c r="P37" t="n">
-        <v>0.3661</v>
+        <v>0.3238</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SVM_RBF</t>
+          <t>KNN</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.9032101966333258</v>
+        <v>0.9205603346469882</v>
       </c>
       <c r="E38" t="n">
-        <v>0.00242878605028493</v>
+        <v>0.003541831237419791</v>
       </c>
       <c r="F38" t="n">
-        <v>0.7582709660512823</v>
+        <v>0.7755728698719533</v>
       </c>
       <c r="G38" t="n">
-        <v>0.004171604488190237</v>
+        <v>0.005642045979370998</v>
       </c>
       <c r="H38" t="n">
-        <v>0.7225322042312822</v>
+        <v>0.8330307606902737</v>
       </c>
       <c r="I38" t="n">
-        <v>0.7979907928504441</v>
+        <v>0.7256528731751095</v>
       </c>
       <c r="J38" t="n">
-        <v>448.563</v>
+        <v>6.912</v>
       </c>
       <c r="K38" t="n">
-        <v>0.9126</v>
+        <v>0.9273</v>
       </c>
       <c r="L38" t="n">
-        <v>0.7613</v>
+        <v>0.7784</v>
       </c>
       <c r="M38" t="n">
-        <v>0.7163</v>
+        <v>0.8207</v>
       </c>
       <c r="N38" t="n">
-        <v>0.8124</v>
+        <v>0.7402</v>
       </c>
       <c r="O38" t="n">
-        <v>0.6536</v>
+        <v>0.6933</v>
       </c>
       <c r="P38" t="n">
-        <v>0.357</v>
+        <v>0.6479</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SVM_RBF</t>
+          <t>KNN</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.9000351655149885</v>
+        <v>0.9205603346469882</v>
       </c>
       <c r="E39" t="n">
-        <v>0.00386559300205514</v>
+        <v>0.003541831237419791</v>
       </c>
       <c r="F39" t="n">
-        <v>0.7400158105610716</v>
+        <v>0.7755728698719533</v>
       </c>
       <c r="G39" t="n">
-        <v>0.001999545657618309</v>
+        <v>0.005642045979370998</v>
       </c>
       <c r="H39" t="n">
-        <v>0.8241293282827232</v>
+        <v>0.8330307606902737</v>
       </c>
       <c r="I39" t="n">
-        <v>0.6716241595992087</v>
+        <v>0.7256528731751095</v>
       </c>
       <c r="J39" t="n">
-        <v>109.93</v>
+        <v>5.686</v>
       </c>
       <c r="K39" t="n">
-        <v>0.9083</v>
+        <v>0.9273</v>
       </c>
       <c r="L39" t="n">
-        <v>0.7541</v>
+        <v>0.7784</v>
       </c>
       <c r="M39" t="n">
-        <v>0.8293</v>
+        <v>0.8207</v>
       </c>
       <c r="N39" t="n">
-        <v>0.6914</v>
+        <v>0.7402</v>
       </c>
       <c r="O39" t="n">
-        <v>0.665</v>
+        <v>0.6933</v>
       </c>
       <c r="P39" t="n">
-        <v>0.3283</v>
+        <v>0.6479</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ensambles</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Bagging</t>
+          <t>KNN</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2655,43 +2655,43 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.8990202201092504</v>
+        <v>0.9165453449080809</v>
       </c>
       <c r="E40" t="n">
-        <v>0.004263840517042803</v>
+        <v>0.002630592056380005</v>
       </c>
       <c r="F40" t="n">
-        <v>0.7375513828142146</v>
+        <v>0.7610276129677098</v>
       </c>
       <c r="G40" t="n">
-        <v>0.008723856147437736</v>
+        <v>0.003930919350853034</v>
       </c>
       <c r="H40" t="n">
-        <v>0.7015943218934325</v>
+        <v>0.6887434653302952</v>
       </c>
       <c r="I40" t="n">
-        <v>0.7779020332791846</v>
+        <v>0.8503684717731155</v>
       </c>
       <c r="J40" t="n">
-        <v>13.502</v>
+        <v>13.685</v>
       </c>
       <c r="K40" t="n">
-        <v>0.9045</v>
+        <v>0.9235</v>
       </c>
       <c r="L40" t="n">
-        <v>0.7378</v>
+        <v>0.7678</v>
       </c>
       <c r="M40" t="n">
-        <v>0.6812</v>
+        <v>0.6908</v>
       </c>
       <c r="N40" t="n">
-        <v>0.8048</v>
+        <v>0.8643</v>
       </c>
       <c r="O40" t="n">
-        <v>0.6162</v>
+        <v>0.656</v>
       </c>
       <c r="P40" t="n">
-        <v>0.3713</v>
+        <v>0.9113</v>
       </c>
     </row>
     <row r="41">
@@ -2702,52 +2702,52 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LogReg</t>
+          <t>SGDElasticNet</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.8850984813019854</v>
+        <v>0.9080340040199995</v>
       </c>
       <c r="E41" t="n">
-        <v>0.004869039549467532</v>
+        <v>0.003540900512979701</v>
       </c>
       <c r="F41" t="n">
-        <v>0.7215904896594297</v>
+        <v>0.7498507807360217</v>
       </c>
       <c r="G41" t="n">
-        <v>0.00357759049344102</v>
+        <v>0.006027893023129959</v>
       </c>
       <c r="H41" t="n">
-        <v>0.6528527229086913</v>
+        <v>0.6816717829089194</v>
       </c>
       <c r="I41" t="n">
-        <v>0.8067637572084841</v>
+        <v>0.8333322562847802</v>
       </c>
       <c r="J41" t="n">
-        <v>6.807</v>
+        <v>4.623</v>
       </c>
       <c r="K41" t="n">
-        <v>0.8912</v>
+        <v>0.9134</v>
       </c>
       <c r="L41" t="n">
-        <v>0.7288</v>
+        <v>0.755</v>
       </c>
       <c r="M41" t="n">
-        <v>0.653</v>
+        <v>0.6817</v>
       </c>
       <c r="N41" t="n">
-        <v>0.8246</v>
+        <v>0.846</v>
       </c>
       <c r="O41" t="n">
-        <v>0.5974</v>
+        <v>0.6375999999999999</v>
       </c>
       <c r="P41" t="n">
-        <v>0.4183</v>
+        <v>0.383</v>
       </c>
     </row>
     <row r="42">
@@ -2758,108 +2758,108 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LogReg</t>
+          <t>SGDElasticNet</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.8850131604431113</v>
+        <v>0.9058661087149359</v>
       </c>
       <c r="E42" t="n">
-        <v>0.004830727805954928</v>
+        <v>0.004884769542416435</v>
       </c>
       <c r="F42" t="n">
-        <v>0.7236380792058493</v>
+        <v>0.747327937025999</v>
       </c>
       <c r="G42" t="n">
-        <v>0.003262651308187069</v>
+        <v>0.01376937941294494</v>
       </c>
       <c r="H42" t="n">
-        <v>0.6592766700839555</v>
+        <v>0.6852618333117529</v>
       </c>
       <c r="I42" t="n">
-        <v>0.8021871624967385</v>
+        <v>0.8231616598718366</v>
       </c>
       <c r="J42" t="n">
-        <v>6.385</v>
+        <v>0.764</v>
       </c>
       <c r="K42" t="n">
-        <v>0.8911</v>
+        <v>0.9132</v>
       </c>
       <c r="L42" t="n">
-        <v>0.731</v>
+        <v>0.7605</v>
       </c>
       <c r="M42" t="n">
-        <v>0.6581</v>
+        <v>0.7102000000000001</v>
       </c>
       <c r="N42" t="n">
-        <v>0.8221000000000001</v>
+        <v>0.8185</v>
       </c>
       <c r="O42" t="n">
-        <v>0.6016</v>
+        <v>0.6513</v>
       </c>
       <c r="P42" t="n">
-        <v>0.4137</v>
+        <v>0.3624</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.8846695588558642</v>
+        <v>0.9057562632928381</v>
       </c>
       <c r="E43" t="n">
-        <v>0.004505009475381636</v>
+        <v>0.003212375345637456</v>
       </c>
       <c r="F43" t="n">
-        <v>0.7145404289681895</v>
+        <v>0.7493470312335072</v>
       </c>
       <c r="G43" t="n">
-        <v>0.008917274356960362</v>
+        <v>0.006349929513041751</v>
       </c>
       <c r="H43" t="n">
-        <v>0.7652063442951079</v>
+        <v>0.6980245716132399</v>
       </c>
       <c r="I43" t="n">
-        <v>0.6704800916999138</v>
+        <v>0.8090520545643567</v>
       </c>
       <c r="J43" t="n">
-        <v>0.445</v>
+        <v>16.298</v>
       </c>
       <c r="K43" t="n">
-        <v>0.8902</v>
+        <v>0.9072</v>
       </c>
       <c r="L43" t="n">
-        <v>0.7209</v>
+        <v>0.7613</v>
       </c>
       <c r="M43" t="n">
-        <v>0.7578</v>
+        <v>0.7294</v>
       </c>
       <c r="N43" t="n">
-        <v>0.6873</v>
+        <v>0.7961</v>
       </c>
       <c r="O43" t="n">
-        <v>0.6133</v>
+        <v>0.6564</v>
       </c>
       <c r="P43" t="n">
-        <v>0.368</v>
+        <v>0.3845</v>
       </c>
     </row>
     <row r="44">
@@ -2870,52 +2870,52 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LogReg</t>
+          <t>SVM_RBF</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.8845935644281168</v>
+        <v>0.9055556282596344</v>
       </c>
       <c r="E44" t="n">
-        <v>0.004943200072061573</v>
+        <v>0.003415658412659005</v>
       </c>
       <c r="F44" t="n">
-        <v>0.7200656311241855</v>
+        <v>0.7564983454614655</v>
       </c>
       <c r="G44" t="n">
-        <v>0.009654675623845083</v>
+        <v>0.006123515596986275</v>
       </c>
       <c r="H44" t="n">
-        <v>0.7756228114556811</v>
+        <v>0.7119822164425902</v>
       </c>
       <c r="I44" t="n">
-        <v>0.6721329842618973</v>
+        <v>0.8071431744875202</v>
       </c>
       <c r="J44" t="n">
-        <v>5.926</v>
+        <v>112.901</v>
       </c>
       <c r="K44" t="n">
-        <v>0.8911</v>
+        <v>0.9142</v>
       </c>
       <c r="L44" t="n">
-        <v>0.7222</v>
+        <v>0.7623</v>
       </c>
       <c r="M44" t="n">
-        <v>0.7658</v>
+        <v>0.7079</v>
       </c>
       <c r="N44" t="n">
-        <v>0.6833</v>
+        <v>0.8256</v>
       </c>
       <c r="O44" t="n">
-        <v>0.6163999999999999</v>
+        <v>0.653</v>
       </c>
       <c r="P44" t="n">
-        <v>0.365</v>
+        <v>0.3252</v>
       </c>
     </row>
     <row r="45">
@@ -2926,52 +2926,52 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SVM_lineal</t>
+          <t>SGDElasticNet</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.8843576981597293</v>
+        <v>0.9051599001258989</v>
       </c>
       <c r="E45" t="n">
-        <v>0.004359519374954015</v>
+        <v>0.003946958430842508</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7255033237336189</v>
+        <v>0.7393836496871475</v>
       </c>
       <c r="G45" t="n">
-        <v>0.006104318062521838</v>
+        <v>0.007832908049006399</v>
       </c>
       <c r="H45" t="n">
-        <v>0.664561018718131</v>
+        <v>0.7825349652936302</v>
       </c>
       <c r="I45" t="n">
-        <v>0.7990083613971797</v>
+        <v>0.7017556429939472</v>
       </c>
       <c r="J45" t="n">
-        <v>222.988</v>
+        <v>0.822</v>
       </c>
       <c r="K45" t="n">
-        <v>0.8894</v>
+        <v>0.9069</v>
       </c>
       <c r="L45" t="n">
-        <v>0.7307</v>
+        <v>0.7494</v>
       </c>
       <c r="M45" t="n">
-        <v>0.6602</v>
+        <v>0.8022</v>
       </c>
       <c r="N45" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.7030999999999999</v>
       </c>
       <c r="O45" t="n">
-        <v>0.6018</v>
+        <v>0.6552</v>
       </c>
       <c r="P45" t="n">
-        <v>0.3695</v>
+        <v>0.3398</v>
       </c>
     </row>
     <row r="46">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2991,43 +2991,43 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.8843344284988561</v>
+        <v>0.9038660096861791</v>
       </c>
       <c r="E46" t="n">
-        <v>0.004410697646695203</v>
+        <v>0.00580205681122376</v>
       </c>
       <c r="F46" t="n">
-        <v>0.7251676987783179</v>
+        <v>0.7359116552775953</v>
       </c>
       <c r="G46" t="n">
-        <v>0.00612483718205405</v>
+        <v>0.007200138561096124</v>
       </c>
       <c r="H46" t="n">
-        <v>0.6614818404456562</v>
+        <v>0.6491643590957055</v>
       </c>
       <c r="I46" t="n">
-        <v>0.8026950178157295</v>
+        <v>0.849860858790049</v>
       </c>
       <c r="J46" t="n">
-        <v>2.828</v>
+        <v>3.093</v>
       </c>
       <c r="K46" t="n">
-        <v>0.8898</v>
+        <v>0.9001</v>
       </c>
       <c r="L46" t="n">
-        <v>0.7287</v>
+        <v>0.7337</v>
       </c>
       <c r="M46" t="n">
-        <v>0.6556999999999999</v>
+        <v>0.6777</v>
       </c>
       <c r="N46" t="n">
-        <v>0.82</v>
+        <v>0.7997</v>
       </c>
       <c r="O46" t="n">
-        <v>0.5981</v>
+        <v>0.6103</v>
       </c>
       <c r="P46" t="n">
-        <v>0.4163</v>
+        <v>0.6812</v>
       </c>
     </row>
     <row r="47">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LDA</t>
+          <t>SVM_RBF</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3047,99 +3047,99 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.8843329932241243</v>
+        <v>0.9032101966333258</v>
       </c>
       <c r="E47" t="n">
-        <v>0.004412754167309445</v>
+        <v>0.00242878605028493</v>
       </c>
       <c r="F47" t="n">
-        <v>0.7249502786152631</v>
+        <v>0.7582709660512823</v>
       </c>
       <c r="G47" t="n">
-        <v>0.00626459617405727</v>
+        <v>0.004171604488190237</v>
       </c>
       <c r="H47" t="n">
-        <v>0.6599831817691921</v>
+        <v>0.7225322042312822</v>
       </c>
       <c r="I47" t="n">
-        <v>0.8043477488204299</v>
+        <v>0.7979907928504441</v>
       </c>
       <c r="J47" t="n">
-        <v>3.107</v>
+        <v>448.563</v>
       </c>
       <c r="K47" t="n">
-        <v>0.8898</v>
+        <v>0.9126</v>
       </c>
       <c r="L47" t="n">
-        <v>0.728</v>
+        <v>0.7613</v>
       </c>
       <c r="M47" t="n">
-        <v>0.6538</v>
+        <v>0.7163</v>
       </c>
       <c r="N47" t="n">
-        <v>0.821</v>
+        <v>0.8124</v>
       </c>
       <c r="O47" t="n">
-        <v>0.5966</v>
+        <v>0.6536</v>
       </c>
       <c r="P47" t="n">
-        <v>0.4215</v>
+        <v>0.357</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SVM_lineal</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.8839391384077853</v>
+        <v>0.9026765293335541</v>
       </c>
       <c r="E48" t="n">
-        <v>0.00432949259336935</v>
+        <v>0.004878767896935301</v>
       </c>
       <c r="F48" t="n">
-        <v>0.7266021910022269</v>
+        <v>0.7361697829446927</v>
       </c>
       <c r="G48" t="n">
-        <v>0.005461443680121344</v>
+        <v>0.01112601087569545</v>
       </c>
       <c r="H48" t="n">
-        <v>0.6664119892739955</v>
+        <v>0.7754078384204025</v>
       </c>
       <c r="I48" t="n">
-        <v>0.7990086845117457</v>
+        <v>0.7015024827315458</v>
       </c>
       <c r="J48" t="n">
-        <v>313.818</v>
+        <v>2.588</v>
       </c>
       <c r="K48" t="n">
-        <v>0.8892</v>
+        <v>0.9109</v>
       </c>
       <c r="L48" t="n">
-        <v>0.7322</v>
+        <v>0.7374000000000001</v>
       </c>
       <c r="M48" t="n">
-        <v>0.6627</v>
+        <v>0.8228</v>
       </c>
       <c r="N48" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.668</v>
       </c>
       <c r="O48" t="n">
-        <v>0.6042999999999999</v>
+        <v>0.6441</v>
       </c>
       <c r="P48" t="n">
-        <v>0.4181</v>
+        <v>0.373</v>
       </c>
     </row>
     <row r="49">
@@ -3150,7 +3150,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SVM_lineal</t>
+          <t>SVM_RBF</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3159,155 +3159,155 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.8829966625011728</v>
+        <v>0.9000351655149885</v>
       </c>
       <c r="E49" t="n">
-        <v>0.004634565943259712</v>
+        <v>0.00386559300205514</v>
       </c>
       <c r="F49" t="n">
-        <v>0.7198124238707404</v>
+        <v>0.7400158105610716</v>
       </c>
       <c r="G49" t="n">
-        <v>0.008186755279267368</v>
+        <v>0.001999545657618309</v>
       </c>
       <c r="H49" t="n">
-        <v>0.7781570502099299</v>
+        <v>0.8241293282827232</v>
       </c>
       <c r="I49" t="n">
-        <v>0.6698444445701002</v>
+        <v>0.6716241595992087</v>
       </c>
       <c r="J49" t="n">
-        <v>196.844</v>
+        <v>109.93</v>
       </c>
       <c r="K49" t="n">
-        <v>0.8898</v>
+        <v>0.9083</v>
       </c>
       <c r="L49" t="n">
-        <v>0.7236</v>
+        <v>0.7541</v>
       </c>
       <c r="M49" t="n">
-        <v>0.773</v>
+        <v>0.8293</v>
       </c>
       <c r="N49" t="n">
-        <v>0.6802</v>
+        <v>0.6914</v>
       </c>
       <c r="O49" t="n">
-        <v>0.6194</v>
+        <v>0.665</v>
       </c>
       <c r="P49" t="n">
-        <v>0.3656</v>
+        <v>0.3283</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Árboles</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>KNN</t>
+          <t>DecisionTree</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.882694998686515</v>
+        <v>0.8999538184092056</v>
       </c>
       <c r="E50" t="n">
-        <v>0.002130639582092924</v>
+        <v>0.003311414395632856</v>
       </c>
       <c r="F50" t="n">
-        <v>0.6997490594988964</v>
+        <v>0.7329380126007593</v>
       </c>
       <c r="G50" t="n">
-        <v>0.01068499371652188</v>
+        <v>0.009663686372255531</v>
       </c>
       <c r="H50" t="n">
-        <v>0.7841276548612377</v>
+        <v>0.6545947385865329</v>
       </c>
       <c r="I50" t="n">
-        <v>0.6319578076999817</v>
+        <v>0.8347279496522884</v>
       </c>
       <c r="J50" t="n">
-        <v>8.791</v>
+        <v>2.813</v>
       </c>
       <c r="K50" t="n">
-        <v>0.8932</v>
+        <v>0.9133</v>
       </c>
       <c r="L50" t="n">
-        <v>0.7244</v>
+        <v>0.7453</v>
       </c>
       <c r="M50" t="n">
-        <v>0.7939000000000001</v>
+        <v>0.6617</v>
       </c>
       <c r="N50" t="n">
-        <v>0.666</v>
+        <v>0.8531</v>
       </c>
       <c r="O50" t="n">
-        <v>0.624</v>
+        <v>0.6201</v>
       </c>
       <c r="P50" t="n">
-        <v>0.7551</v>
+        <v>0.4213</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>KNN</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.882694998686515</v>
+        <v>0.8997149781030049</v>
       </c>
       <c r="E51" t="n">
-        <v>0.002130639582092924</v>
+        <v>0.004231156829102635</v>
       </c>
       <c r="F51" t="n">
-        <v>0.6997490594988964</v>
+        <v>0.7267192283247618</v>
       </c>
       <c r="G51" t="n">
-        <v>0.01068499371652188</v>
+        <v>0.01577460752560449</v>
       </c>
       <c r="H51" t="n">
-        <v>0.7841276548612377</v>
+        <v>0.7864884931006975</v>
       </c>
       <c r="I51" t="n">
-        <v>0.6319578076999817</v>
+        <v>0.6805268544554671</v>
       </c>
       <c r="J51" t="n">
-        <v>5.851</v>
+        <v>18.532</v>
       </c>
       <c r="K51" t="n">
-        <v>0.8932</v>
+        <v>0.8977000000000001</v>
       </c>
       <c r="L51" t="n">
-        <v>0.7244</v>
+        <v>0.7271</v>
       </c>
       <c r="M51" t="n">
-        <v>0.7939000000000001</v>
+        <v>0.7665999999999999</v>
       </c>
       <c r="N51" t="n">
-        <v>0.666</v>
+        <v>0.6914</v>
       </c>
       <c r="O51" t="n">
-        <v>0.624</v>
+        <v>0.6223</v>
       </c>
       <c r="P51" t="n">
-        <v>0.7551</v>
+        <v>0.7409</v>
       </c>
     </row>
     <row r="52">
@@ -3318,52 +3318,52 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.8823283036933158</v>
+        <v>0.8904495092967712</v>
       </c>
       <c r="E52" t="n">
-        <v>0.004433864610869031</v>
+        <v>0.0127432871352812</v>
       </c>
       <c r="F52" t="n">
-        <v>0.7116779433492628</v>
+        <v>0.7261581011517647</v>
       </c>
       <c r="G52" t="n">
-        <v>0.008854312699560982</v>
+        <v>0.01875638316318416</v>
       </c>
       <c r="H52" t="n">
-        <v>0.7700876878870713</v>
+        <v>0.6575439998429703</v>
       </c>
       <c r="I52" t="n">
-        <v>0.661835807717753</v>
+        <v>0.8189757914489345</v>
       </c>
       <c r="J52" t="n">
-        <v>0.525</v>
+        <v>2.54</v>
       </c>
       <c r="K52" t="n">
-        <v>0.8887</v>
+        <v>0.8931</v>
       </c>
       <c r="L52" t="n">
-        <v>0.7205</v>
+        <v>0.7156</v>
       </c>
       <c r="M52" t="n">
-        <v>0.7651</v>
+        <v>0.6206</v>
       </c>
       <c r="N52" t="n">
-        <v>0.6807</v>
+        <v>0.8449</v>
       </c>
       <c r="O52" t="n">
-        <v>0.6142</v>
+        <v>0.5709</v>
       </c>
       <c r="P52" t="n">
-        <v>0.3681</v>
+        <v>0.8991</v>
       </c>
     </row>
     <row r="53">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LDA</t>
+          <t>LogReg</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3383,43 +3383,43 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.8823181498223265</v>
+        <v>0.8850984813019854</v>
       </c>
       <c r="E53" t="n">
-        <v>0.004427890999659801</v>
+        <v>0.004869039549467532</v>
       </c>
       <c r="F53" t="n">
-        <v>0.714960077452233</v>
+        <v>0.7215904896594297</v>
       </c>
       <c r="G53" t="n">
-        <v>0.01017420782088104</v>
+        <v>0.00357759049344102</v>
       </c>
       <c r="H53" t="n">
-        <v>0.7588041582669012</v>
+        <v>0.6528527229086913</v>
       </c>
       <c r="I53" t="n">
-        <v>0.6762009966468786</v>
+        <v>0.8067637572084841</v>
       </c>
       <c r="J53" t="n">
-        <v>5.021</v>
+        <v>6.807</v>
       </c>
       <c r="K53" t="n">
-        <v>0.8887</v>
+        <v>0.8912</v>
       </c>
       <c r="L53" t="n">
-        <v>0.726</v>
+        <v>0.7288</v>
       </c>
       <c r="M53" t="n">
-        <v>0.7599</v>
+        <v>0.653</v>
       </c>
       <c r="N53" t="n">
-        <v>0.695</v>
+        <v>0.8246</v>
       </c>
       <c r="O53" t="n">
-        <v>0.6197</v>
+        <v>0.5974</v>
       </c>
       <c r="P53" t="n">
-        <v>0.37</v>
+        <v>0.4183</v>
       </c>
     </row>
     <row r="54">
@@ -3430,108 +3430,108 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LDA</t>
+          <t>LogReg</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.8823181498223265</v>
+        <v>0.8850131604431113</v>
       </c>
       <c r="E54" t="n">
-        <v>0.004427890999659801</v>
+        <v>0.004830727805954928</v>
       </c>
       <c r="F54" t="n">
-        <v>0.714960077452233</v>
+        <v>0.7236380792058493</v>
       </c>
       <c r="G54" t="n">
-        <v>0.01017420782088104</v>
+        <v>0.003262651308187069</v>
       </c>
       <c r="H54" t="n">
-        <v>0.7588041582669012</v>
+        <v>0.6592766700839555</v>
       </c>
       <c r="I54" t="n">
-        <v>0.6762009966468786</v>
+        <v>0.8021871624967385</v>
       </c>
       <c r="J54" t="n">
-        <v>4.421</v>
+        <v>6.385</v>
       </c>
       <c r="K54" t="n">
-        <v>0.8887</v>
+        <v>0.8911</v>
       </c>
       <c r="L54" t="n">
-        <v>0.726</v>
+        <v>0.731</v>
       </c>
       <c r="M54" t="n">
-        <v>0.7599</v>
+        <v>0.6581</v>
       </c>
       <c r="N54" t="n">
-        <v>0.695</v>
+        <v>0.8221000000000001</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6197</v>
+        <v>0.6016</v>
       </c>
       <c r="P54" t="n">
-        <v>0.37</v>
+        <v>0.4137</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>KNN</t>
+          <t>LogReg</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.8765323572985777</v>
+        <v>0.8845935644281168</v>
       </c>
       <c r="E55" t="n">
-        <v>0.00189915403459892</v>
+        <v>0.004943200072061573</v>
       </c>
       <c r="F55" t="n">
-        <v>0.6987706725914837</v>
+        <v>0.7200656311241855</v>
       </c>
       <c r="G55" t="n">
-        <v>0.001943441120628007</v>
+        <v>0.009654675623845083</v>
       </c>
       <c r="H55" t="n">
-        <v>0.6173106039839186</v>
+        <v>0.7756228114556811</v>
       </c>
       <c r="I55" t="n">
-        <v>0.8051105415319345</v>
+        <v>0.6721329842618973</v>
       </c>
       <c r="J55" t="n">
-        <v>11.26</v>
+        <v>5.926</v>
       </c>
       <c r="K55" t="n">
-        <v>0.8859</v>
+        <v>0.8911</v>
       </c>
       <c r="L55" t="n">
-        <v>0.7116</v>
+        <v>0.7222</v>
       </c>
       <c r="M55" t="n">
-        <v>0.6268</v>
+        <v>0.7658</v>
       </c>
       <c r="N55" t="n">
-        <v>0.8231000000000001</v>
+        <v>0.6833</v>
       </c>
       <c r="O55" t="n">
-        <v>0.5683</v>
+        <v>0.6163999999999999</v>
       </c>
       <c r="P55" t="n">
-        <v>0.9792</v>
+        <v>0.365</v>
       </c>
     </row>
     <row r="56">
@@ -3542,287 +3542,287 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>SVM_lineal</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.8741241306358422</v>
+        <v>0.8843576981597293</v>
       </c>
       <c r="E56" t="n">
-        <v>0.005511197211547377</v>
+        <v>0.004359519374954015</v>
       </c>
       <c r="F56" t="n">
-        <v>0.7131382162666238</v>
+        <v>0.7255033237336189</v>
       </c>
       <c r="G56" t="n">
-        <v>0.003093239870022109</v>
+        <v>0.006104318062521838</v>
       </c>
       <c r="H56" t="n">
-        <v>0.6465284319982184</v>
+        <v>0.664561018718131</v>
       </c>
       <c r="I56" t="n">
-        <v>0.7962127741728066</v>
+        <v>0.7990083613971797</v>
       </c>
       <c r="J56" t="n">
-        <v>4.999</v>
+        <v>222.988</v>
       </c>
       <c r="K56" t="n">
-        <v>0.8861</v>
+        <v>0.8894</v>
       </c>
       <c r="L56" t="n">
-        <v>0.7187</v>
+        <v>0.7307</v>
       </c>
       <c r="M56" t="n">
-        <v>0.6447000000000001</v>
+        <v>0.6602</v>
       </c>
       <c r="N56" t="n">
-        <v>0.8119</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="O56" t="n">
-        <v>0.5826</v>
+        <v>0.6018</v>
       </c>
       <c r="P56" t="n">
-        <v>0.8823</v>
+        <v>0.3695</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>LDA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.8717836427536556</v>
+        <v>0.8843329932241243</v>
       </c>
       <c r="E57" t="n">
-        <v>0.009995687307184685</v>
+        <v>0.004412754167309445</v>
       </c>
       <c r="F57" t="n">
-        <v>0.6921021153867956</v>
+        <v>0.7249502786152631</v>
       </c>
       <c r="G57" t="n">
-        <v>0.01337270905694012</v>
+        <v>0.00626459617405727</v>
       </c>
       <c r="H57" t="n">
-        <v>0.6256096023463031</v>
+        <v>0.6599831817691921</v>
       </c>
       <c r="I57" t="n">
-        <v>0.7749780887934983</v>
+        <v>0.8043477488204299</v>
       </c>
       <c r="J57" t="n">
-        <v>7.777</v>
+        <v>3.107</v>
       </c>
       <c r="K57" t="n">
-        <v>0.8709</v>
+        <v>0.8898</v>
       </c>
       <c r="L57" t="n">
-        <v>0.7074</v>
+        <v>0.728</v>
       </c>
       <c r="M57" t="n">
-        <v>0.6578000000000001</v>
+        <v>0.6538</v>
       </c>
       <c r="N57" t="n">
-        <v>0.7651</v>
+        <v>0.821</v>
       </c>
       <c r="O57" t="n">
-        <v>0.5731000000000001</v>
+        <v>0.5966</v>
       </c>
       <c r="P57" t="n">
-        <v>0.5194</v>
+        <v>0.4215</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>BernoulliNB</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.8661494164195437</v>
+        <v>0.8841486780021585</v>
       </c>
       <c r="E58" t="n">
-        <v>0.00671958876914109</v>
+        <v>0.005967561688845147</v>
       </c>
       <c r="F58" t="n">
-        <v>0.6941913512113745</v>
+        <v>0.7209644616533369</v>
       </c>
       <c r="G58" t="n">
-        <v>0.01006942602794927</v>
+        <v>0.005524605109551882</v>
       </c>
       <c r="H58" t="n">
-        <v>0.730478335432205</v>
+        <v>0.7132624744453478</v>
       </c>
       <c r="I58" t="n">
-        <v>0.6628575767538456</v>
+        <v>0.7289597892000572</v>
       </c>
       <c r="J58" t="n">
-        <v>5.234</v>
+        <v>0.331</v>
       </c>
       <c r="K58" t="n">
-        <v>0.8783</v>
+        <v>0.8875</v>
       </c>
       <c r="L58" t="n">
-        <v>0.7084</v>
+        <v>0.7239</v>
       </c>
       <c r="M58" t="n">
-        <v>0.7476</v>
+        <v>0.701</v>
       </c>
       <c r="N58" t="n">
-        <v>0.6731</v>
+        <v>0.7483</v>
       </c>
       <c r="O58" t="n">
-        <v>0.5966</v>
+        <v>0.6044</v>
       </c>
       <c r="P58" t="n">
-        <v>0.9693000000000001</v>
+        <v>0.4728</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Lineales</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>BernoulliNB</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.863202763096637</v>
+        <v>0.8841486780021585</v>
       </c>
       <c r="E59" t="n">
-        <v>0.01055555723602859</v>
+        <v>0.005967561688845147</v>
       </c>
       <c r="F59" t="n">
-        <v>0.6959085906644356</v>
+        <v>0.7209644616533369</v>
       </c>
       <c r="G59" t="n">
-        <v>0.01949689649156733</v>
+        <v>0.005524605109551882</v>
       </c>
       <c r="H59" t="n">
-        <v>0.6248996621655765</v>
+        <v>0.7132624744453478</v>
       </c>
       <c r="I59" t="n">
-        <v>0.7878241545909329</v>
+        <v>0.7289597892000572</v>
       </c>
       <c r="J59" t="n">
-        <v>5.38</v>
+        <v>0.286</v>
       </c>
       <c r="K59" t="n">
-        <v>0.87</v>
+        <v>0.8875</v>
       </c>
       <c r="L59" t="n">
-        <v>0.6918</v>
+        <v>0.7239</v>
       </c>
       <c r="M59" t="n">
-        <v>0.6133999999999999</v>
+        <v>0.701</v>
       </c>
       <c r="N59" t="n">
-        <v>0.7931</v>
+        <v>0.7483</v>
       </c>
       <c r="O59" t="n">
-        <v>0.5401</v>
+        <v>0.6044</v>
       </c>
       <c r="P59" t="n">
-        <v>1.2521</v>
+        <v>0.4728</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>SVM_lineal</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>smote</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.8629433668971502</v>
+        <v>0.8839391384077853</v>
       </c>
       <c r="E60" t="n">
-        <v>0.01097309759275986</v>
+        <v>0.00432949259336935</v>
       </c>
       <c r="F60" t="n">
-        <v>0.6667710064068929</v>
+        <v>0.7266021910022269</v>
       </c>
       <c r="G60" t="n">
-        <v>0.01894239180031032</v>
+        <v>0.005461443680121344</v>
       </c>
       <c r="H60" t="n">
-        <v>0.7489098357091311</v>
+        <v>0.6664119892739955</v>
       </c>
       <c r="I60" t="n">
-        <v>0.6031004458173224</v>
+        <v>0.7990086845117457</v>
       </c>
       <c r="J60" t="n">
-        <v>2.818</v>
+        <v>313.818</v>
       </c>
       <c r="K60" t="n">
-        <v>0.8725000000000001</v>
+        <v>0.8892</v>
       </c>
       <c r="L60" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.7322</v>
       </c>
       <c r="M60" t="n">
-        <v>0.7973</v>
+        <v>0.6627</v>
       </c>
       <c r="N60" t="n">
-        <v>0.6019</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="O60" t="n">
-        <v>0.5804</v>
+        <v>0.6042999999999999</v>
       </c>
       <c r="P60" t="n">
-        <v>0.4128</v>
+        <v>0.4181</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Árboles</t>
+          <t>Otros</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>DecisionTree</t>
+          <t>BernoulliNB</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3831,54 +3831,54 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.8587799720113086</v>
+        <v>0.8834440899523732</v>
       </c>
       <c r="E61" t="n">
-        <v>0.01610594815560971</v>
+        <v>0.006091741210467352</v>
       </c>
       <c r="F61" t="n">
-        <v>0.6897703602942326</v>
+        <v>0.719159332462157</v>
       </c>
       <c r="G61" t="n">
-        <v>0.02240601914767313</v>
+        <v>0.006442997893351844</v>
       </c>
       <c r="H61" t="n">
-        <v>0.6453804703360848</v>
+        <v>0.6634652662075602</v>
       </c>
       <c r="I61" t="n">
-        <v>0.7414163403882708</v>
+        <v>0.7851511893443279</v>
       </c>
       <c r="J61" t="n">
-        <v>10.122</v>
+        <v>2.696</v>
       </c>
       <c r="K61" t="n">
-        <v>0.8703</v>
+        <v>0.8868</v>
       </c>
       <c r="L61" t="n">
-        <v>0.7007</v>
+        <v>0.7212</v>
       </c>
       <c r="M61" t="n">
-        <v>0.6685</v>
+        <v>0.6536999999999999</v>
       </c>
       <c r="N61" t="n">
-        <v>0.7361</v>
+        <v>0.8043</v>
       </c>
       <c r="O61" t="n">
-        <v>0.5684</v>
+        <v>0.5884</v>
       </c>
       <c r="P61" t="n">
-        <v>0.4682</v>
+        <v>0.5286</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GaussianNB</t>
+          <t>Perceptron</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3887,43 +3887,43 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.8529648303212822</v>
+        <v>0.8832410336398798</v>
       </c>
       <c r="E62" t="n">
-        <v>0.004837693111059647</v>
+        <v>0.007139590517034026</v>
       </c>
       <c r="F62" t="n">
-        <v>0.6866545587450258</v>
+        <v>0.7158664191688076</v>
       </c>
       <c r="G62" t="n">
-        <v>0.006819172052795935</v>
+        <v>0.00986043738027908</v>
       </c>
       <c r="H62" t="n">
-        <v>0.62191207990752</v>
+        <v>0.6531384758078419</v>
       </c>
       <c r="I62" t="n">
-        <v>0.7665892268757002</v>
+        <v>0.7923979220502264</v>
       </c>
       <c r="J62" t="n">
-        <v>1.141</v>
+        <v>8.765000000000001</v>
       </c>
       <c r="K62" t="n">
-        <v>0.8609</v>
+        <v>0.8915</v>
       </c>
       <c r="L62" t="n">
-        <v>0.7023</v>
+        <v>0.7274</v>
       </c>
       <c r="M62" t="n">
-        <v>0.6292</v>
+        <v>0.6519</v>
       </c>
       <c r="N62" t="n">
-        <v>0.7946</v>
+        <v>0.8226</v>
       </c>
       <c r="O62" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.5953000000000001</v>
       </c>
       <c r="P62" t="n">
-        <v>0.596</v>
+        <v>0.4494</v>
       </c>
     </row>
     <row r="63">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Perceptron</t>
+          <t>SVM_lineal</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3943,43 +3943,43 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.8488396124380351</v>
+        <v>0.8829966625011728</v>
       </c>
       <c r="E63" t="n">
-        <v>0.008353262699786791</v>
+        <v>0.004634565943259712</v>
       </c>
       <c r="F63" t="n">
-        <v>0.5867712130180907</v>
+        <v>0.7198124238707404</v>
       </c>
       <c r="G63" t="n">
-        <v>0.03591590599266724</v>
+        <v>0.008186755279267368</v>
       </c>
       <c r="H63" t="n">
-        <v>0.8153247288753673</v>
+        <v>0.7781570502099299</v>
       </c>
       <c r="I63" t="n">
-        <v>0.4600861423432753</v>
+        <v>0.6698444445701002</v>
       </c>
       <c r="J63" t="n">
-        <v>5.942</v>
+        <v>196.844</v>
       </c>
       <c r="K63" t="n">
-        <v>0.8433</v>
+        <v>0.8898</v>
       </c>
       <c r="L63" t="n">
-        <v>0.4452</v>
+        <v>0.7236</v>
       </c>
       <c r="M63" t="n">
-        <v>0.7376</v>
+        <v>0.773</v>
       </c>
       <c r="N63" t="n">
-        <v>0.3188</v>
+        <v>0.6802</v>
       </c>
       <c r="O63" t="n">
-        <v>0.3262</v>
+        <v>0.6194</v>
       </c>
       <c r="P63" t="n">
-        <v>0.4671</v>
+        <v>0.3656</v>
       </c>
     </row>
     <row r="64">
@@ -3990,63 +3990,63 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Perceptron</t>
+          <t>LDA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>balanced</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.848525965825041</v>
+        <v>0.8823181498223265</v>
       </c>
       <c r="E64" t="n">
-        <v>0.004987952975853188</v>
+        <v>0.004427890999659801</v>
       </c>
       <c r="F64" t="n">
-        <v>0.4857065282087784</v>
+        <v>0.714960077452233</v>
       </c>
       <c r="G64" t="n">
-        <v>0.03844693262637554</v>
+        <v>0.01017420782088104</v>
       </c>
       <c r="H64" t="n">
-        <v>0.7984896368776917</v>
+        <v>0.7588041582669012</v>
       </c>
       <c r="I64" t="n">
-        <v>0.3517710313251493</v>
+        <v>0.6762009966468786</v>
       </c>
       <c r="J64" t="n">
-        <v>6.822</v>
+        <v>4.421</v>
       </c>
       <c r="K64" t="n">
-        <v>0.8502</v>
+        <v>0.8887</v>
       </c>
       <c r="L64" t="n">
-        <v>0.4648</v>
+        <v>0.726</v>
       </c>
       <c r="M64" t="n">
-        <v>0.7408</v>
+        <v>0.7599</v>
       </c>
       <c r="N64" t="n">
-        <v>0.3386</v>
+        <v>0.695</v>
       </c>
       <c r="O64" t="n">
-        <v>0.3445</v>
+        <v>0.6197</v>
       </c>
       <c r="P64" t="n">
-        <v>0.4769</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>GaussianNB</t>
+          <t>LDA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -4055,99 +4055,99 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.8469549915922656</v>
+        <v>0.8823181498223265</v>
       </c>
       <c r="E65" t="n">
-        <v>0.005025110789714717</v>
+        <v>0.004427890999659801</v>
       </c>
       <c r="F65" t="n">
-        <v>0.6755478540484857</v>
+        <v>0.714960077452233</v>
       </c>
       <c r="G65" t="n">
-        <v>0.009749038200879478</v>
+        <v>0.01017420782088104</v>
       </c>
       <c r="H65" t="n">
-        <v>0.6768333234912273</v>
+        <v>0.7588041582669012</v>
       </c>
       <c r="I65" t="n">
-        <v>0.6745464885120654</v>
+        <v>0.6762009966468786</v>
       </c>
       <c r="J65" t="n">
-        <v>4.106</v>
+        <v>5.021</v>
       </c>
       <c r="K65" t="n">
-        <v>0.8547</v>
+        <v>0.8887</v>
       </c>
       <c r="L65" t="n">
-        <v>0.6875</v>
+        <v>0.726</v>
       </c>
       <c r="M65" t="n">
-        <v>0.6855</v>
+        <v>0.7599</v>
       </c>
       <c r="N65" t="n">
-        <v>0.6894</v>
+        <v>0.695</v>
       </c>
       <c r="O65" t="n">
-        <v>0.5577</v>
+        <v>0.6197</v>
       </c>
       <c r="P65" t="n">
-        <v>0.5866</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Otros</t>
+          <t>Lineales</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>GaussianNB</t>
+          <t>Perceptron</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>balanced</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.8469549915922656</v>
+        <v>0.869424006109857</v>
       </c>
       <c r="E66" t="n">
-        <v>0.005025110789714717</v>
+        <v>0.0218725251244608</v>
       </c>
       <c r="F66" t="n">
-        <v>0.6755478540484857</v>
+        <v>0.6319948658525671</v>
       </c>
       <c r="G66" t="n">
-        <v>0.009749038200879478</v>
+        <v>0.0390039191867483</v>
       </c>
       <c r="H66" t="n">
-        <v>0.6768333234912273</v>
+        <v>0.7954658103754625</v>
       </c>
       <c r="I66" t="n">
-        <v>0.6745464885120654</v>
+        <v>0.5260559585960995</v>
       </c>
       <c r="J66" t="n">
-        <v>4.989</v>
+        <v>8.106</v>
       </c>
       <c r="K66" t="n">
-        <v>0.8547</v>
+        <v>0.8597</v>
       </c>
       <c r="L66" t="n">
-        <v>0.6875</v>
+        <v>0.4465</v>
       </c>
       <c r="M66" t="n">
-        <v>0.6855</v>
+        <v>0.716</v>
       </c>
       <c r="N66" t="n">
-        <v>0.6894</v>
+        <v>0.3244</v>
       </c>
       <c r="O66" t="n">
-        <v>0.5577</v>
+        <v>0.323</v>
       </c>
       <c r="P66" t="n">
-        <v>0.5866</v>
+        <v>0.4591</v>
       </c>
     </row>
     <row r="67">
@@ -4163,47 +4163,47 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>smote</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.8426267344924778</v>
+        <v>0.8692919612377658</v>
       </c>
       <c r="E67" t="n">
-        <v>0.01293406320725295</v>
+        <v>0.009158002606966488</v>
       </c>
       <c r="F67" t="n">
-        <v>0.6701084643253468</v>
+        <v>0.6224816539270621</v>
       </c>
       <c r="G67" t="n">
-        <v>0.02069116428210701</v>
+        <v>0.04430817190313216</v>
       </c>
       <c r="H67" t="n">
-        <v>0.599996685635648</v>
+        <v>0.8075223176092313</v>
       </c>
       <c r="I67" t="n">
-        <v>0.7598566502228279</v>
+        <v>0.5100422391516304</v>
       </c>
       <c r="J67" t="n">
-        <v>5.913</v>
+        <v>5.042</v>
       </c>
       <c r="K67" t="n">
-        <v>0.8339</v>
+        <v>0.855</v>
       </c>
       <c r="L67" t="n">
-        <v>0.6731</v>
+        <v>0.5841</v>
       </c>
       <c r="M67" t="n">
-        <v>0.6014</v>
+        <v>0.7534</v>
       </c>
       <c r="N67" t="n">
-        <v>0.7641</v>
+        <v>0.4769</v>
       </c>
       <c r="O67" t="n">
-        <v>0.514</v>
+        <v>0.4621</v>
       </c>
       <c r="P67" t="n">
-        <v>0.5302</v>
+        <v>0.4427</v>
       </c>
     </row>
     <row r="68">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>BernoulliNB</t>
+          <t>GaussianNB</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4223,43 +4223,43 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.829684692324722</v>
+        <v>0.8668456883336573</v>
       </c>
       <c r="E68" t="n">
-        <v>0.006262854064077574</v>
+        <v>0.006217101728968266</v>
       </c>
       <c r="F68" t="n">
-        <v>0.6321575370589098</v>
+        <v>0.717791033451685</v>
       </c>
       <c r="G68" t="n">
-        <v>0.007691049953674287</v>
+        <v>0.01318829961392401</v>
       </c>
       <c r="H68" t="n">
-        <v>0.5372733918142222</v>
+        <v>0.6792291950196319</v>
       </c>
       <c r="I68" t="n">
-        <v>0.767988232167509</v>
+        <v>0.7611215629697783</v>
       </c>
       <c r="J68" t="n">
-        <v>2.167</v>
+        <v>1.685</v>
       </c>
       <c r="K68" t="n">
-        <v>0.8466</v>
+        <v>0.8695000000000001</v>
       </c>
       <c r="L68" t="n">
-        <v>0.6541</v>
+        <v>0.7174</v>
       </c>
       <c r="M68" t="n">
-        <v>0.5563</v>
+        <v>0.6726</v>
       </c>
       <c r="N68" t="n">
-        <v>0.7936</v>
+        <v>0.7687</v>
       </c>
       <c r="O68" t="n">
-        <v>0.4728</v>
+        <v>0.5893</v>
       </c>
       <c r="P68" t="n">
-        <v>0.5427</v>
+        <v>1.068</v>
       </c>
     </row>
     <row r="69">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>BernoulliNB</t>
+          <t>GaussianNB</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -4279,43 +4279,43 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.8288793012322191</v>
+        <v>0.8655993475111388</v>
       </c>
       <c r="E69" t="n">
-        <v>0.005686738806756303</v>
+        <v>0.005162576597865669</v>
       </c>
       <c r="F69" t="n">
-        <v>0.6340433055736778</v>
+        <v>0.6934780834307281</v>
       </c>
       <c r="G69" t="n">
-        <v>0.006963301764446998</v>
+        <v>0.01257431233199609</v>
       </c>
       <c r="H69" t="n">
-        <v>0.6106528813202753</v>
+        <v>0.699957726433367</v>
       </c>
       <c r="I69" t="n">
-        <v>0.6594188299860011</v>
+        <v>0.6872589464364907</v>
       </c>
       <c r="J69" t="n">
-        <v>0.143</v>
+        <v>3.378</v>
       </c>
       <c r="K69" t="n">
-        <v>0.8459</v>
+        <v>0.8682</v>
       </c>
       <c r="L69" t="n">
-        <v>0.6562</v>
+        <v>0.6951000000000001</v>
       </c>
       <c r="M69" t="n">
-        <v>0.6313</v>
+        <v>0.6983</v>
       </c>
       <c r="N69" t="n">
-        <v>0.6833</v>
+        <v>0.6919</v>
       </c>
       <c r="O69" t="n">
-        <v>0.5061</v>
+        <v>0.5699</v>
       </c>
       <c r="P69" t="n">
-        <v>0.4687</v>
+        <v>1.0734</v>
       </c>
     </row>
     <row r="70">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>BernoulliNB</t>
+          <t>GaussianNB</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -4335,43 +4335,43 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.8288793012322191</v>
+        <v>0.8655993475111388</v>
       </c>
       <c r="E70" t="n">
-        <v>0.005686738806756303</v>
+        <v>0.005162576597865669</v>
       </c>
       <c r="F70" t="n">
-        <v>0.6340433055736778</v>
+        <v>0.6934780834307281</v>
       </c>
       <c r="G70" t="n">
-        <v>0.006963301764446998</v>
+        <v>0.01257431233199609</v>
       </c>
       <c r="H70" t="n">
-        <v>0.6106528813202753</v>
+        <v>0.699957726433367</v>
       </c>
       <c r="I70" t="n">
-        <v>0.6594188299860011</v>
+        <v>0.6872589464364907</v>
       </c>
       <c r="J70" t="n">
-        <v>0.256</v>
+        <v>5.223</v>
       </c>
       <c r="K70" t="n">
-        <v>0.8459</v>
+        <v>0.8682</v>
       </c>
       <c r="L70" t="n">
-        <v>0.6562</v>
+        <v>0.6951000000000001</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6313</v>
+        <v>0.6983</v>
       </c>
       <c r="N70" t="n">
-        <v>0.6833</v>
+        <v>0.6919</v>
       </c>
       <c r="O70" t="n">
-        <v>0.5061</v>
+        <v>0.5699</v>
       </c>
       <c r="P70" t="n">
-        <v>0.4687</v>
+        <v>1.0734</v>
       </c>
     </row>
   </sheetData>

</xml_diff>